<commit_message>
Giai đoạn 2- Điều chỉnh Flow
</commit_message>
<xml_diff>
--- a/server/dataset/cancuoc/question.xlsx
+++ b/server/dataset/cancuoc/question.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\HTML CSS JAVASCRIPT\CCHC\server\dataset\cancuoc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A10349E1-CE35-4C6C-88D5-07DA09906E24}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E8C484A-289F-4DAD-BB9A-C224E13F8845}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,13 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
-  <si>
-    <t>Question</t>
-  </si>
-  <si>
-    <t>Anwser</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Làm Căn cước khi nào có</t>
   </si>
@@ -43,6 +37,22 @@
   </si>
   <si>
     <t>Bạn có thể làm Căn cước tại các xã trong phạm vi huyện bạn thường trú nhé</t>
+  </si>
+  <si>
+    <t>question</t>
+  </si>
+  <si>
+    <t>anwser</t>
+  </si>
+  <si>
+    <t>Hỗ trợ tôi cấp Căn cước, CCCD</t>
+  </si>
+  <si>
+    <t>Tôi có thể hỗ trợ ạn cấp Căn cước:
+Bạn có thể cung cấp thông tin về:
+Bạn đã có thẻ Căn cước chưa, hay là chỉ là Căn cước công dân
+Bạn dưới 14 tuổi hay trên 14 tuổi
+Tôi sẽ giúp bạn nộp hồ sơ cấp Căn cước phù hợp và cấp cho bạn trong thời gian sớm nhất có thể.</t>
   </si>
 </sst>
 </file>
@@ -384,36 +394,40 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30" style="2" customWidth="1"/>
-    <col min="2" max="2" width="40.77734375" style="2" customWidth="1"/>
+    <col min="2" max="2" width="45.44140625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="3"/>

</xml_diff>